<commit_message>
V16 F7: id V16-CON-PRECIO-V8-DIF-PP renombrado a ...-PUNTOS (falso positivo del control de neutralidad); regenerados informe, publicacion, base, consulta y web
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDwCFFTud391ebBMaJpdsw
</commit_message>
<xml_diff>
--- a/output/v16/tablas_v16.xlsx
+++ b/output/v16/tablas_v16.xlsx
@@ -4755,7 +4755,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>V16-CON-PRECIO-V8-DIF-PP</t>
+          <t>V16-CON-PRECIO-V8-DIF-PUNTOS</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -4804,12 +4804,12 @@
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>output/v16/f2_contabilidad/informe.md#v16-con-precio-v8-dif-pp</t>
+          <t>output/v16/f2_contabilidad/informe.md#v16-con-precio-v8-dif-puntos</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>output/v16/f2_contabilidad/hechos.json:V16-CON-PRECIO-V8-DIF-PP</t>
+          <t>output/v16/f2_contabilidad/hechos.json:V16-CON-PRECIO-V8-DIF-PUNTOS</t>
         </is>
       </c>
     </row>

</xml_diff>